<commit_message>
sync: update attendance records with full 4-slot punches
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,12 +58,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00CF1322"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="001D39C4"/>
       <sz val="10"/>
     </font>
@@ -74,7 +68,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -97,12 +91,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F6FFED"/>
         <bgColor rgb="00F6FFED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF1F0"/>
-        <bgColor rgb="00FFF1F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -199,10 +187,7 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -635,7 +620,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 12:57:25</t>
+          <t>2026-09-09 14:07:44</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -793,17 +778,17 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
@@ -867,17 +852,17 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M7" s="14" t="n">
@@ -959,12 +944,12 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>unpaid_leave</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
         <is>
-          <t>曠工/缺勤 (Vắng mặt/Nghỉ không phép)</t>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P8" s="10" t="inlineStr"/>
@@ -1015,17 +1000,17 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M9" s="14" t="n">
@@ -1089,17 +1074,17 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
@@ -1163,17 +1148,17 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M11" s="14" t="n">
@@ -1237,17 +1222,17 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
@@ -1311,17 +1296,17 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M13" s="14" t="n">
@@ -1385,17 +1370,17 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
@@ -1459,17 +1444,17 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M15" s="14" t="n">
@@ -1533,17 +1518,17 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
@@ -1607,17 +1592,17 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M17" s="14" t="n">
@@ -1681,17 +1666,17 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
@@ -3034,7 +3019,7 @@
           <t>unpaid_leave</t>
         </is>
       </c>
-      <c r="O36" s="17" t="inlineStr">
+      <c r="O36" s="16" t="inlineStr">
         <is>
           <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
@@ -3256,7 +3241,7 @@
           <t>unpaid_leave</t>
         </is>
       </c>
-      <c r="O39" s="17" t="inlineStr">
+      <c r="O39" s="16" t="inlineStr">
         <is>
           <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
@@ -3478,7 +3463,7 @@
           <t>unpaid_leave</t>
         </is>
       </c>
-      <c r="O42" s="17" t="inlineStr">
+      <c r="O42" s="16" t="inlineStr">
         <is>
           <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
@@ -3552,7 +3537,7 @@
           <t>unpaid_leave</t>
         </is>
       </c>
-      <c r="O43" s="17" t="inlineStr">
+      <c r="O43" s="16" t="inlineStr">
         <is>
           <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
@@ -4514,7 +4499,7 @@
           <t>early_leave</t>
         </is>
       </c>
-      <c r="O56" s="18" t="inlineStr">
+      <c r="O56" s="17" t="inlineStr">
         <is>
           <t>早退 (Về sớm)</t>
         </is>
@@ -5613,72 +5598,72 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 12:57:25</t>
+          <t>2026-09-09 14:07:44</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>項次
 STT</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>員工工號
 Mã NV</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>打卡機號
 Mã máy</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>員工姓名
 Họ và tên</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>部門
 Bộ phận</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>職務
 Chức vụ</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>出勤天數
 Số ngày</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>累計工時(h)
 Tổng giờ</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>正常天數
 Bình thường</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>遲到次數
 Đi muộn</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>缺勤/請假(天)
 Nghỉ/Vắng</t>
@@ -5717,7 +5702,7 @@
       <c r="G5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="19" t="n">
         <v>40</v>
       </c>
       <c r="I5" s="14" t="n">
@@ -5762,7 +5747,7 @@
       <c r="G6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="20" t="n">
         <v>40</v>
       </c>
       <c r="I6" s="8" t="n">
@@ -5807,7 +5792,7 @@
       <c r="G7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="19" t="n">
         <v>40</v>
       </c>
       <c r="I7" s="14" t="n">
@@ -5852,7 +5837,7 @@
       <c r="G8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="20" t="n">
         <v>32</v>
       </c>
       <c r="I8" s="8" t="n">
@@ -5897,7 +5882,7 @@
       <c r="G9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="19" t="n">
         <v>40</v>
       </c>
       <c r="I9" s="14" t="n">
@@ -5942,7 +5927,7 @@
       <c r="G10" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="20" t="n">
         <v>40</v>
       </c>
       <c r="I10" s="8" t="n">
@@ -5987,7 +5972,7 @@
       <c r="G11" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="19" t="n">
         <v>35.9</v>
       </c>
       <c r="I11" s="14" t="n">
@@ -6032,7 +6017,7 @@
       <c r="G12" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="21" t="n">
+      <c r="H12" s="20" t="n">
         <v>40</v>
       </c>
       <c r="I12" s="8" t="n">
@@ -6077,7 +6062,7 @@
       <c r="G13" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="20" t="n">
+      <c r="H13" s="19" t="n">
         <v>40</v>
       </c>
       <c r="I13" s="14" t="n">
@@ -6122,7 +6107,7 @@
       <c r="G14" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="21" t="n">
+      <c r="H14" s="20" t="n">
         <v>32</v>
       </c>
       <c r="I14" s="8" t="n">
@@ -6167,7 +6152,7 @@
       <c r="G15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="20" t="n">
+      <c r="H15" s="19" t="n">
         <v>31.91</v>
       </c>
       <c r="I15" s="14" t="n">
@@ -6212,7 +6197,7 @@
       <c r="G16" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="20" t="n">
         <v>30.36</v>
       </c>
       <c r="I16" s="8" t="n">
@@ -6257,7 +6242,7 @@
       <c r="G17" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="H17" s="20" t="n">
+      <c r="H17" s="19" t="n">
         <v>40</v>
       </c>
       <c r="I17" s="14" t="n">

</xml_diff>

<commit_message>
fix: correctly place morning half-day punch in lunch_out instead of check_out
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 14:07:44</t>
+          <t>2026-09-09 14:42:36</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -3220,17 +3220,17 @@
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K39" s="11" t="inlineStr">
+      <c r="L39" s="11" t="inlineStr">
         <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="L39" s="11" t="inlineStr">
-        <is>
-          <t>11:31</t>
         </is>
       </c>
       <c r="M39" s="14" t="n">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 14:07:44</t>
+          <t>2026-09-09 14:42:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: push 2026-09-09 attendance records to GitHub Pages
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -620,7 +620,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 14:42:36</t>
+          <t>2026-09-10 09:57:57</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>65 筆</t>
+          <t>78 筆</t>
         </is>
       </c>
     </row>
@@ -763,32 +763,32 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>07:25</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
@@ -837,32 +837,32 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M7" s="14" t="n">
@@ -911,45 +911,45 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0</v>
+        <v>7.98</v>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O8" s="16" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P8" s="10" t="inlineStr"/>
@@ -985,17 +985,17 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
@@ -1059,22 +1059,22 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1133,27 +1133,27 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="L11" s="11" t="inlineStr">
@@ -1207,27 +1207,27 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1281,17 +1281,17 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="J13" s="11" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
@@ -1355,32 +1355,32 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>07:25</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
@@ -1429,17 +1429,17 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>07:25</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
@@ -1503,45 +1503,45 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O16" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O16" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P16" s="10" t="inlineStr"/>
@@ -1577,27 +1577,27 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
@@ -1651,22 +1651,22 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>週二 (Thứ Ba)</t>
+          <t>週三 (Thứ Tư)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
@@ -1725,17 +1725,17 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M19" s="14" t="n">
@@ -1799,32 +1799,32 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
@@ -1873,45 +1873,45 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M21" s="14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O21" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O21" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P21" s="15" t="inlineStr"/>
@@ -1947,17 +1947,17 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -2021,12 +2021,12 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L23" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M23" s="14" t="n">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
@@ -2169,32 +2169,32 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M25" s="14" t="n">
@@ -2243,17 +2243,17 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -2317,17 +2317,17 @@
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="J27" s="11" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L27" s="11" t="inlineStr">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2465,17 +2465,17 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>07:23</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
@@ -2539,17 +2539,17 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
@@ -2613,32 +2613,32 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>週一 (Thứ Hai)</t>
+          <t>週二 (Thứ Ba)</t>
         </is>
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L31" s="11" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="M31" s="14" t="n">
@@ -2687,17 +2687,17 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2707,12 +2707,12 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="M32" s="8" t="n">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
@@ -2776,17 +2776,17 @@
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>11:37</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>17:17</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="M33" s="14" t="n">
@@ -2835,27 +2835,27 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="M34" s="8" t="n">
-        <v>7.91</v>
+        <v>8</v>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
@@ -2909,17 +2909,17 @@
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr">
@@ -2929,12 +2929,12 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L35" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M35" s="14" t="n">
@@ -2983,45 +2983,45 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O36" s="16" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P36" s="10" t="inlineStr"/>
@@ -3057,27 +3057,27 @@
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L37" s="11" t="inlineStr">
@@ -3131,22 +3131,22 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="M38" s="8" t="n">
@@ -3205,45 +3205,45 @@
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L39" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M39" s="14" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O39" s="16" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P39" s="15" t="inlineStr"/>
@@ -3279,27 +3279,27 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="J41" s="11" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="L41" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M41" s="14" t="n">
@@ -3427,45 +3427,45 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M42" s="8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O42" s="16" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P42" s="10" t="inlineStr"/>
@@ -3501,45 +3501,45 @@
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="L43" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M43" s="14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O43" s="16" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P43" s="15" t="inlineStr"/>
@@ -3575,32 +3575,32 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>週六 (Thứ Bảy)</t>
+          <t>週一 (Thứ Hai)</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="M44" s="8" t="n">
@@ -3649,17 +3649,17 @@
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J45" s="11" t="inlineStr">
@@ -3669,12 +3669,12 @@
       </c>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="L45" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M45" s="14" t="n">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -3738,17 +3738,17 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="M46" s="8" t="n">
@@ -3797,27 +3797,27 @@
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="L47" s="11" t="inlineStr">
@@ -3826,7 +3826,7 @@
         </is>
       </c>
       <c r="M47" s="14" t="n">
-        <v>8</v>
+        <v>7.91</v>
       </c>
       <c r="N47" s="11" t="inlineStr">
         <is>
@@ -3871,17 +3871,17 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3891,12 +3891,12 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M48" s="8" t="n">
@@ -3945,45 +3945,45 @@
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L49" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M49" s="14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O49" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O49" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P49" s="15" t="inlineStr"/>
@@ -4019,27 +4019,27 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="L50" s="5" t="inlineStr">
@@ -4093,22 +4093,22 @@
       </c>
       <c r="G51" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="K51" s="11" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="L51" s="11" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="M51" s="14" t="n">
@@ -4167,45 +4167,45 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>13:06</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M52" s="8" t="n">
-        <v>7.9</v>
+        <v>4</v>
       </c>
       <c r="N52" s="5" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O52" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O52" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P52" s="10" t="inlineStr"/>
@@ -4241,27 +4241,27 @@
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
@@ -4335,12 +4335,12 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M54" s="8" t="n">
@@ -4389,45 +4389,45 @@
       </c>
       <c r="G55" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M55" s="14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O55" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O55" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P55" s="15" t="inlineStr"/>
@@ -4463,45 +4463,45 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M56" s="8" t="n">
-        <v>6.36</v>
+        <v>0</v>
       </c>
       <c r="N56" s="5" t="inlineStr">
         <is>
-          <t>early_leave</t>
-        </is>
-      </c>
-      <c r="O56" s="17" t="inlineStr">
-        <is>
-          <t>早退 (Về sớm)</t>
+          <t>unpaid_leave</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>事假/無薪假 (Nghỉ không lương)</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr"/>
@@ -4537,22 +4537,22 @@
       </c>
       <c r="G57" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>週五 (Thứ Sáu)</t>
+          <t>週六 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>11:35</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K57" s="11" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M57" s="14" t="n">
@@ -4611,17 +4611,17 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -4685,12 +4685,12 @@
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I59" s="11" t="inlineStr">
@@ -4700,12 +4700,12 @@
       </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="L59" s="11" t="inlineStr">
@@ -4759,27 +4759,27 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>12:52</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -4833,17 +4833,17 @@
       </c>
       <c r="G61" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L61" s="11" t="inlineStr">
@@ -4907,27 +4907,27 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -4981,17 +4981,17 @@
       </c>
       <c r="G63" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H63" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L63" s="11" t="inlineStr">
@@ -5055,32 +5055,32 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="M64" s="8" t="n">
@@ -5129,17 +5129,17 @@
       </c>
       <c r="G65" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H65" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>13:06</t>
         </is>
       </c>
       <c r="L65" s="11" t="inlineStr">
@@ -5158,7 +5158,7 @@
         </is>
       </c>
       <c r="M65" s="14" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="N65" s="11" t="inlineStr">
         <is>
@@ -5203,32 +5203,32 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="M66" s="8" t="n">
@@ -5277,17 +5277,17 @@
       </c>
       <c r="G67" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H67" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
@@ -5297,12 +5297,12 @@
       </c>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>12:59</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="M67" s="14" t="n">
@@ -5351,17 +5351,17 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:52</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr">
@@ -5425,45 +5425,45 @@
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="M69" s="14" t="n">
-        <v>8</v>
+        <v>6.36</v>
       </c>
       <c r="N69" s="11" t="inlineStr">
         <is>
-          <t>normal</t>
-        </is>
-      </c>
-      <c r="O69" s="9" t="inlineStr">
-        <is>
-          <t>正常 (Bình thường)</t>
+          <t>early_leave</t>
+        </is>
+      </c>
+      <c r="O69" s="17" t="inlineStr">
+        <is>
+          <t>早退 (Về sớm)</t>
         </is>
       </c>
       <c r="P69" s="15" t="inlineStr"/>
@@ -5499,22 +5499,22 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>週四 (Thứ Năm)</t>
+          <t>週五 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="M70" s="8" t="n">
@@ -5541,6 +5541,968 @@
         </is>
       </c>
       <c r="P70" s="10" t="inlineStr"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="11" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>EMP-002</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>Dương Thị Nam Hoài</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H71" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I71" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J71" s="11" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K71" s="11" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="L71" s="11" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="M71" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N71" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O71" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P71" s="15" t="inlineStr"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>EMP-001</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Phan Thị Hải</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>現場主管</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="M72" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O72" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P72" s="10" t="inlineStr"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>EMP-011</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Hoàng Thị Nga</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H73" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I73" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J73" s="11" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="K73" s="11" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="L73" s="11" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="M73" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N73" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O73" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P73" s="15" t="inlineStr"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>EMP-003</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Trần Thị Ly</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>倉管</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M74" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N74" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O74" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P74" s="10" t="inlineStr"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>EMP-004</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>Lê Thị Mai</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H75" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="L75" s="11" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="M75" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N75" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O75" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P75" s="15" t="inlineStr"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>EMP-005</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Hoàng Thị Thảo</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M76" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N76" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O76" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P76" s="10" t="inlineStr"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>EMP-006</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Chu Thị Thúy Quỳnh</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽辦公室</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>辦公室（財務及人事）</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="L77" s="11" t="inlineStr">
+        <is>
+          <t>17:06</t>
+        </is>
+      </c>
+      <c r="M77" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N77" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O77" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P77" s="15" t="inlineStr"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>EMP-007</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Sái Văn Quân</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M78" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N78" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O78" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P78" s="10" t="inlineStr"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>EMP-008</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Phùng Văn Tuyền</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G79" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="K79" s="11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="L79" s="11" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M79" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N79" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O79" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P79" s="15" t="inlineStr"/>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>EMP-009</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Hoàng Thị Chất</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="M80" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N80" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P80" s="10" t="inlineStr"/>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>EMP-010</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr">
+        <is>
+          <t>Đào Thanh Long</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F81" s="11" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G81" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J81" s="11" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="L81" s="11" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M81" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N81" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O81" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P81" s="15" t="inlineStr"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>EMP-012</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Lương Thị Thêm</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>萬和富壽現場</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>現場普工</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="M82" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N82" s="5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P82" s="10" t="inlineStr"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>EMP-013</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="inlineStr">
+        <is>
+          <t>Lê Thị Thủy</t>
+        </is>
+      </c>
+      <c r="E83" s="11" t="inlineStr">
+        <is>
+          <t>萬和富壽辦公室</t>
+        </is>
+      </c>
+      <c r="F83" s="11" t="inlineStr">
+        <is>
+          <t>辦公室（生管）</t>
+        </is>
+      </c>
+      <c r="G83" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H83" s="11" t="inlineStr">
+        <is>
+          <t>週四 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="I83" s="11" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J83" s="11" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="K83" s="11" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="L83" s="11" t="inlineStr">
+        <is>
+          <t>17:06</t>
+        </is>
+      </c>
+      <c r="M83" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="N83" s="11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O83" s="9" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
+        </is>
+      </c>
+      <c r="P83" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5598,7 +6560,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-09 14:42:36</t>
+          <t>2026-09-10 09:57:57</t>
         </is>
       </c>
     </row>
@@ -5700,13 +6662,13 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5" s="14" t="n">
         <v>0</v>
@@ -5745,13 +6707,13 @@
         </is>
       </c>
       <c r="G6" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>0</v>
@@ -5790,13 +6752,13 @@
         </is>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J7" s="14" t="n">
         <v>0</v>
@@ -5835,13 +6797,13 @@
         </is>
       </c>
       <c r="G8" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="I8" s="8" t="n">
         <v>5</v>
-      </c>
-      <c r="H8" s="20" t="n">
-        <v>32</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>4</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>0</v>
@@ -5880,13 +6842,13 @@
         </is>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H9" s="19" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J9" s="14" t="n">
         <v>0</v>
@@ -5925,13 +6887,13 @@
         </is>
       </c>
       <c r="G10" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>0</v>
@@ -5970,13 +6932,13 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I11" s="14" t="n">
         <v>5</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>4</v>
       </c>
       <c r="J11" s="14" t="n">
         <v>0</v>
@@ -6015,13 +6977,13 @@
         </is>
       </c>
       <c r="G12" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>0</v>
@@ -6060,13 +7022,13 @@
         </is>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13" s="14" t="n">
         <v>0</v>
@@ -6105,7 +7067,7 @@
         </is>
       </c>
       <c r="G14" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H14" s="20" t="n">
         <v>32</v>
@@ -6117,7 +7079,7 @@
         <v>0</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -6150,13 +7112,13 @@
         </is>
       </c>
       <c r="G15" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>39.89</v>
+      </c>
+      <c r="I15" s="14" t="n">
         <v>5</v>
-      </c>
-      <c r="H15" s="19" t="n">
-        <v>31.91</v>
-      </c>
-      <c r="I15" s="14" t="n">
-        <v>4</v>
       </c>
       <c r="J15" s="14" t="n">
         <v>0</v>
@@ -6195,13 +7157,13 @@
         </is>
       </c>
       <c r="G16" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>30.36</v>
+        <v>38.36</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>0</v>
@@ -6240,13 +7202,13 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J17" s="14" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
data: update attendance records up to 2026-09-25
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -650,7 +650,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-28 07:54:52</t>
+          <t>2026-09-28 08:24:10</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -9928,12 +9928,12 @@
       </c>
       <c r="N129" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O129" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O129" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P129" s="16" t="inlineStr"/>
@@ -10072,16 +10072,16 @@
         </is>
       </c>
       <c r="M131" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N131" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O131" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O131" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P131" s="16" t="inlineStr"/>
@@ -10150,12 +10150,12 @@
       </c>
       <c r="N132" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O132" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O132" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P132" s="10" t="inlineStr"/>
@@ -10224,12 +10224,12 @@
       </c>
       <c r="N133" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O133" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O133" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P133" s="16" t="inlineStr"/>
@@ -10298,12 +10298,12 @@
       </c>
       <c r="N134" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O134" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O134" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P134" s="10" t="inlineStr"/>
@@ -10368,16 +10368,16 @@
         </is>
       </c>
       <c r="M135" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N135" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O135" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O135" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P135" s="16" t="inlineStr"/>
@@ -10442,16 +10442,16 @@
         </is>
       </c>
       <c r="M136" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N136" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O136" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O136" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P136" s="10" t="inlineStr"/>
@@ -10516,16 +10516,16 @@
         </is>
       </c>
       <c r="M137" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N137" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O137" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O137" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P137" s="16" t="inlineStr"/>
@@ -10590,16 +10590,16 @@
         </is>
       </c>
       <c r="M138" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N138" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O138" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O138" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P138" s="10" t="inlineStr"/>
@@ -10664,16 +10664,16 @@
         </is>
       </c>
       <c r="M139" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N139" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O139" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O139" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P139" s="16" t="inlineStr"/>
@@ -10738,16 +10738,16 @@
         </is>
       </c>
       <c r="M140" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N140" s="5" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O140" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O140" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P140" s="10" t="inlineStr"/>
@@ -10812,16 +10812,16 @@
         </is>
       </c>
       <c r="M141" s="14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N141" s="11" t="inlineStr">
         <is>
-          <t>unpaid_leave</t>
-        </is>
-      </c>
-      <c r="O141" s="9" t="inlineStr">
-        <is>
-          <t>事假/無薪假 (Nghỉ không lương)</t>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="O141" s="15" t="inlineStr">
+        <is>
+          <t>正常 (Bình thường)</t>
         </is>
       </c>
       <c r="P141" s="16" t="inlineStr"/>
@@ -17764,7 +17764,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-28 07:54:52</t>
+          <t>2026-09-28 08:24:10</t>
         </is>
       </c>
     </row>
@@ -17917,13 +17917,13 @@
         <v>104</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -17962,13 +17962,13 @@
         <v>137.96</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J7" s="14" t="n">
         <v>1</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -18007,13 +18007,13 @@
         <v>124</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -18052,13 +18052,13 @@
         <v>132</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J9" s="14" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -18094,16 +18094,16 @@
         <v>18</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>135.88</v>
+        <v>139.88</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -18139,16 +18139,16 @@
         <v>9</v>
       </c>
       <c r="H11" s="21" t="n">
-        <v>51.9</v>
+        <v>55.9</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11" s="14" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -18184,16 +18184,16 @@
         <v>18</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>129.96</v>
+        <v>133.96</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -18229,16 +18229,16 @@
         <v>18</v>
       </c>
       <c r="H13" s="21" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J13" s="14" t="n">
         <v>0</v>
       </c>
       <c r="K13" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -18274,16 +18274,16 @@
         <v>10</v>
       </c>
       <c r="H14" s="22" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -18319,16 +18319,16 @@
         <v>18</v>
       </c>
       <c r="H15" s="21" t="n">
-        <v>111.83</v>
+        <v>115.83</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J15" s="14" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -18364,16 +18364,16 @@
         <v>18</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>82.31999999999999</v>
+        <v>86.31999999999999</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
@@ -18409,16 +18409,16 @@
         <v>18</v>
       </c>
       <c r="H17" s="21" t="n">
-        <v>119.96</v>
+        <v>123.96</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J17" s="14" t="n">
         <v>0</v>
       </c>
       <c r="K17" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">

</xml_diff>